<commit_message>
feat: add persistent deck-editing consumables
</commit_message>
<xml_diff>
--- a/CardPG_GameData_organized.xlsx
+++ b/CardPG_GameData_organized.xlsx
@@ -25321,7 +25321,7 @@
       </c>
       <c r="E5" s="20" t="inlineStr">
         <is>
-          <t>Duplicate a card.</t>
+          <t>Copy one card's effective suit, rank, enhancement and permanent attack bonus into a new card ID. Combat: select a hand card; copy enters discard. Outside combat: select any owned card; copy enters the next encounter deck.</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr">
@@ -25344,10 +25344,14 @@
       </c>
       <c r="J5" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="K5" s="20" t="n"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>Run-persistent; three nonstacking backpack slots; only stable unblocked interaction states.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="12.75" customHeight="1" s="14">
       <c r="A6" s="16" t="inlineStr">
@@ -25372,7 +25376,7 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>Destroy up to 2 cards.</t>
+          <t>Permanently destroy one or two distinct cards; at least one deck card must survive. Combat targets must be in hand; outside combat targets may be any owned cards. Cancel without consuming.</t>
         </is>
       </c>
       <c r="F6" s="16" t="inlineStr">
@@ -25395,10 +25399,14 @@
       </c>
       <c r="J6" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="K6" s="20" t="n"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>Run-persistent; three nonstacking backpack slots; only stable unblocked interaction states.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="12.75" customHeight="1" s="14">
       <c r="A7" s="16" t="inlineStr">
@@ -25933,7 +25941,7 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Change a card's suit to Spades.</t>
+          <t>Change one card's effective suit to Spade per charge; same-suit target spends no charge. Three charges remain in one backpack slot until exhausted. Combat: hand target; outside combat: any owned card.</t>
         </is>
       </c>
       <c r="F17" s="16" t="inlineStr">
@@ -25956,10 +25964,14 @@
       </c>
       <c r="J17" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="K17" s="20" t="n"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>Run-persistent; three nonstacking backpack slots; only stable unblocked interaction states.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="12.75" customHeight="1" s="14">
       <c r="A18" s="16" t="inlineStr">
@@ -25984,7 +25996,7 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>Change a card's suit to Hearts.</t>
+          <t>Change one card's effective suit to Heart per charge; same-suit target spends no charge. Three charges remain in one backpack slot until exhausted. Combat: hand target; outside combat: any owned card.</t>
         </is>
       </c>
       <c r="F18" s="16" t="inlineStr">
@@ -26007,10 +26019,14 @@
       </c>
       <c r="J18" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="K18" s="20" t="n"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>Run-persistent; three nonstacking backpack slots; only stable unblocked interaction states.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="12.75" customHeight="1" s="14">
       <c r="A19" s="16" t="inlineStr">
@@ -26035,7 +26051,7 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Change a card's suit to Clubs.</t>
+          <t>Change one card's effective suit to Club per charge; same-suit target spends no charge. Three charges remain in one backpack slot until exhausted. Combat: hand target; outside combat: any owned card.</t>
         </is>
       </c>
       <c r="F19" s="16" t="inlineStr">
@@ -26058,10 +26074,14 @@
       </c>
       <c r="J19" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="K19" s="20" t="n"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>Run-persistent; three nonstacking backpack slots; only stable unblocked interaction states.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="12.75" customHeight="1" s="14">
       <c r="A20" s="16" t="inlineStr">
@@ -26086,7 +26106,7 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>Change a card's suit to Diamonds.</t>
+          <t>Change one card's effective suit to Diamond per charge; same-suit target spends no charge. Three charges remain in one backpack slot until exhausted. Combat: hand target; outside combat: any owned card.</t>
         </is>
       </c>
       <c r="F20" s="16" t="inlineStr">
@@ -26109,10 +26129,14 @@
       </c>
       <c r="J20" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="K20" s="20" t="n"/>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>Run-persistent; three nonstacking backpack slots; only stable unblocked interaction states.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="12.75" customHeight="1" s="14">
       <c r="A21" s="16" t="inlineStr">

</xml_diff>

<commit_message>
feat: implement milestone 2 artifact upgrades
</commit_message>
<xml_diff>
--- a/CardPG_GameData_organized.xlsx
+++ b/CardPG_GameData_organized.xlsx
@@ -3958,12 +3958,12 @@
       </c>
       <c r="G23" s="20" t="inlineStr">
         <is>
-          <t>Counterattack after blocking; deal double damage when block value exceeds 150% of the enemy attack.</t>
+          <t>After blocking, retaliate against the attacker for damage actually blocked. If committed block is strictly greater than 150% of incoming attack, deal double the blocked damage.</t>
         </is>
       </c>
       <c r="H23" s="16" t="inlineStr">
         <is>
-          <t>Blocked damage</t>
+          <t>Blocked damage; ×2 above 150%</t>
         </is>
       </c>
       <c r="I23" s="16" t="inlineStr">
@@ -3983,7 +3983,7 @@
       </c>
       <c r="L23" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="M23" s="20" t="n"/>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="G26" s="20" t="inlineStr">
         <is>
-          <t>Multiply total damage.</t>
+          <t>Club card attacks deal double final damage after flat bonuses, before enemy mitigation.</t>
         </is>
       </c>
       <c r="H26" s="16" t="inlineStr">
@@ -4182,7 +4182,7 @@
       </c>
       <c r="L26" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="M26" s="20" t="n"/>
@@ -4224,11 +4224,13 @@
       </c>
       <c r="G27" s="20" t="inlineStr">
         <is>
-          <t>Heal HP; gain Gold while below 50% HP.</t>
-        </is>
-      </c>
-      <c r="H27" s="16" t="n">
-        <v>3</v>
+          <t>Playing a Heart heals 3 HP. If HP was below 50% immediately before the heal, gain 3 Gold.</t>
+        </is>
+      </c>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>+3 HP; +3 Gold below 50%</t>
+        </is>
       </c>
       <c r="I27" s="16" t="inlineStr">
         <is>
@@ -4247,7 +4249,7 @@
       </c>
       <c r="L27" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="M27" s="20" t="n"/>
@@ -4289,11 +4291,13 @@
       </c>
       <c r="G28" s="20" t="inlineStr">
         <is>
-          <t>Draw cards.</t>
-        </is>
-      </c>
-      <c r="H28" s="16" t="n">
-        <v>2</v>
+          <t>Playing a Diamond draws 2 cards through the normal draw path.</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>2 cards</t>
+        </is>
       </c>
       <c r="I28" s="16" t="inlineStr">
         <is>
@@ -4312,7 +4316,7 @@
       </c>
       <c r="L28" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="M28" s="20" t="n"/>
@@ -4419,11 +4423,13 @@
       </c>
       <c r="G30" s="20" t="inlineStr">
         <is>
-          <t>Increase hand size, but take 50% additional damage.</t>
-        </is>
-      </c>
-      <c r="H30" s="16" t="n">
-        <v>3</v>
+          <t>Gain 3 hand slots and take 1.5× incoming attack damage, rounded up once after other incoming modifiers and before block. Event HP costs are unaffected.</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>+3 slots; ×1.5 incoming attack</t>
+        </is>
       </c>
       <c r="I30" s="16" t="inlineStr">
         <is>
@@ -4442,7 +4448,7 @@
       </c>
       <c r="L30" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="M30" s="20" t="n"/>
@@ -4551,7 +4557,7 @@
       </c>
       <c r="G32" s="20" t="inlineStr">
         <is>
-          <t>Deal 5 additional damage, but take 5 additional damage.</t>
+          <t>Card attacks deal +5 damage; incoming attacks deal +5 damage.</t>
         </is>
       </c>
       <c r="H32" s="16" t="inlineStr">
@@ -4576,7 +4582,7 @@
       </c>
       <c r="L32" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="M32" s="20" t="n"/>
@@ -4618,7 +4624,7 @@
       </c>
       <c r="G33" s="20" t="inlineStr">
         <is>
-          <t>Deal double damage, but take double damage.</t>
+          <t>Card attacks and incoming attacks deal 2× damage. Replaces Common Glass; does not inherit +5 vulnerability.</t>
         </is>
       </c>
       <c r="H33" s="16" t="inlineStr">
@@ -4643,7 +4649,7 @@
       </c>
       <c r="L33" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="M33" s="20" t="n"/>
@@ -4685,12 +4691,12 @@
       </c>
       <c r="G34" s="20" t="inlineStr">
         <is>
-          <t>Deal triple damage.</t>
+          <t>At exactly 1 HP, card attacks deal 3× damage; otherwise card attacks deal normal damage. Replaces Rare Glass and has no inherited vulnerability.</t>
         </is>
       </c>
       <c r="H34" s="16" t="inlineStr">
         <is>
-          <t>×3</t>
+          <t>×3 at 1 HP</t>
         </is>
       </c>
       <c r="I34" s="16" t="inlineStr">
@@ -4710,7 +4716,7 @@
       </c>
       <c r="L34" s="16" t="inlineStr">
         <is>
-          <t>Draft</t>
+          <t>Implemented</t>
         </is>
       </c>
       <c r="M34" s="20" t="n"/>

</xml_diff>